<commit_message>
feat: refactor contests to standalone entities and add cleanup action
Rework contest import/export to use contest title/status/deadline without user/email linkage, and expose contests for the public map panel. Add admin bulk-delete endpoint and UI button to clear all contests from the database when needed.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/frontend/public/samples/contests-import-sample.xlsx
+++ b/frontend/public/samples/contests-import-sample.xlsx
@@ -413,168 +413,141 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>название</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>конкурсы</t>
+          <t>статус</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>дата окончания</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Описание</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Статус</t>
-        </is>
-      </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Срок подачи</t>
+          <t>Формат</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>aabaurina@edu.hse.ru</t>
+          <t>Олимпиада школьников</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Олимпиада школьников ВШЭ</t>
+          <t>Прием заявок</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>до 20 мая</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Очный этап, математика и информатика</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Участник</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>Очно</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>aabaurina@edu.hse.ru</t>
+          <t>Конкурс проектных работ</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Конкурс проектных работ</t>
+          <t>Идет отбор</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>до 28 мая</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Командный проект по анализу данных</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Заявка подана</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>Смешанный</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>aabaurina@edu.hse.ru</t>
+          <t>Региональный трек</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Региональный трек</t>
+          <t>Скоро старт</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Отборочный этап в Нижнем Новгороде</t>
+          <t>с 1 июня</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Участник</t>
+          <t>Отборочный этап</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>Дистанционно</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>neznakomyy.abiturient@example.com</t>
+          <t>Портфолио абитуриента</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Конкурс проектных работ</t>
+          <t>Открыт</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Индивидуальная заявка</t>
+          <t>до 15 июня</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>На рассмотрении</t>
+          <t>Загрузка материалов</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>drugoy.chuzhak@mail.ru</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Региональный трек</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Дистанционный формат</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Участник</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-02-28</t>
+          <t>Онлайн</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add DB-backed contest ordering on map
Load map contests from API with switchable ordering (database order or by parsed deadline date), and store normalized deadline_on in DB via new migration and import parsing updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/frontend/public/samples/contests-import-sample.xlsx
+++ b/frontend/public/samples/contests-import-sample.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -454,10 +457,8 @@
           <t>Прием заявок</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>до 20 мая</t>
-        </is>
+      <c r="C2" s="1" t="n">
+        <v>46162</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -481,10 +482,8 @@
           <t>Идет отбор</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>до 28 мая</t>
-        </is>
+      <c r="C3" s="1" t="n">
+        <v>46170</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -508,10 +507,8 @@
           <t>Скоро старт</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>с 1 июня</t>
-        </is>
+      <c r="C4" s="1" t="n">
+        <v>46174</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -535,10 +532,8 @@
           <t>Открыт</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>до 15 июня</t>
-        </is>
+      <c r="C5" s="1" t="n">
+        <v>46188</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>

</xml_diff>